<commit_message>
do form demografi dewasa done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18740" yWindow="-19340" windowWidth="34560" windowHeight="18900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -483,6 +483,21 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>status_perkawinan</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>rencana_menikah</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>disabilitas</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
@@ -505,11 +520,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Belum Menikah</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Non disabilitas</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Ya,Tidak"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
demografi, kanker usus, tb, hati done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18740" yWindow="-19340" windowWidth="34560" windowHeight="18900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="22500" yWindow="-21000" windowWidth="19200" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -455,9 +455,15 @@
     <col width="11.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="14.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="10.83203125" customWidth="1" style="1" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="1" min="9" max="9"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
+    <col width="21" bestFit="1" customWidth="1" min="10" max="10"/>
     <col width="16" bestFit="1" customWidth="1" min="11" max="11"/>
     <col width="13.5" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="19.5" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="11.5" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="16.5" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="14.5" bestFit="1" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,6 +504,66 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>keluarga_kanker_usus</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>merokok</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>batuk_tidak_sembuh</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>hepatitis_b</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ibu_hepatitis_b</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>seks_bukan_pasangan</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>transfusi_darah</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>hemodialisis</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>pengguna_narkoba</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>odhiv</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>hepatitis_c</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>kolesterol_tinggi</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
@@ -535,21 +601,82 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Ya, kurang dari 2 minggu</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
+    <dataValidation sqref="J2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
skrining perilaku merokok done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AL2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -471,6 +471,14 @@
     <col width="19.1640625" bestFit="1" customWidth="1" min="26" max="26"/>
     <col width="11.5" bestFit="1" customWidth="1" min="27" max="27"/>
     <col width="5.33203125" bestFit="1" customWidth="1" min="28" max="28"/>
+    <col width="25.1640625" bestFit="1" customWidth="1" min="30" max="30"/>
+    <col width="49" bestFit="1" customWidth="1" min="31" max="31"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="32" max="32"/>
+    <col width="13.1640625" bestFit="1" customWidth="1" min="33" max="33"/>
+    <col width="14.5" bestFit="1" customWidth="1" min="34" max="34"/>
+    <col width="23.6640625" bestFit="1" customWidth="1" min="35" max="35"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="36" max="36"/>
+    <col width="23" bestFit="1" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,6 +629,46 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>merokok_setahun_terakhir_b</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>jenis_rokok</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>berapa_tahun</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>berapa_batang</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>pernah_merokok</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>berapa_tahun_sebelumnya</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>kapan_berhenti</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>terpapar_sebulan_terakhir</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
@@ -738,7 +786,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -767,25 +815,62 @@
         </is>
       </c>
       <c r="AD2" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Rokok konvensional (rokok putih, filter, kretek, tingwe, dll)</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>15</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>1 s.d &lt;10 tahun lalu</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
+    <dataValidation sqref="J2 AE2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
     <dataValidation sqref="T2:W2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
skrining mandiri dewasa done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -446,7 +446,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:BD2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1023,34 +1023,7 @@
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Timeout 30000ms exceeded.
-Call log:
-  - waiting for locator("#sq_112i_list [role='option']").filter(has_text="Ya")
-    - locator resolved to &lt;li role="option" tabindex="-1" aria-selected="false" id="sq_112i_listPPV00001265" class="sv-list__item sd-list__item sv-list__item-text--wrap"&gt;…&lt;/li&gt;
-  - attempting click action
-    2 × waiting for element to be visible, enabled and stable
-      - element is visible, enabled and stable
-      - scrolling into view if needed
-      - done scrolling
-      - &lt;div id="sq_112" role="combobox" data-rendered="r" aria-required="true" aria-invalid="false" aria-expanded="false" aria-labelledby="sq_112_ariaTitle" data-name="LPM000002|FRM000169|PPM00000718|text" class="sd-element--with-frame sd-element sd-question sd-row__question sd-question--title-top sd-row__question--small"&gt;…&lt;/div&gt; intercepts pointer events
-    - retrying click action
-    - waiting 20ms
-    - waiting for element to be visible, enabled and stable
-    - element is visible, enabled and stable
-    - scrolling into view if needed
-    - done scrolling
-    - &lt;div id="sq_112" role="combobox" data-rendered="r" aria-required="true" aria-invalid="false" aria-expanded="false" aria-labelledby="sq_112_ariaTitle" data-name="LPM000002|FRM000169|PPM00000718|text" class="sd-element--with-frame sd-element sd-question sd-row__question sd-question--title-top sd-row__question--small"&gt;…&lt;/div&gt; intercepts pointer events
-  2 × retrying click action
-      - waiting 100ms
-      - waiting for element to be visible, enabled and stable
-      - element is not visible
-  57 × retrying click action
-       - waiting 500ms
-       - waiting for element to be visible, enabled and stable
-       - element is not visible
-  - retrying click action
-    - waiting 500ms
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
centang pemeriksaan insya Allah done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3300" yWindow="-21000" windowWidth="19200" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3300" yWindow="-21000" windowWidth="19200" windowHeight="19700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -45,9 +45,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,7 +449,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:BD2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1021,21 +1024,9 @@
       <c r="BC2" t="n">
         <v>20</v>
       </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FAILED: Locator.set_checked: Clicking the checkbox did not change its state
-Call log:
-  - waiting for locator("input#hasil-lab-0-1")
-    - locator resolved to &lt;input checked type="checkbox" id="hasil-lab-0-1" class="peer sr-only"/&gt;
-  - attempting click action
-    - scrolling into view if needed
-    - done scrolling
-    - forcing action
-    - performing click action
-    - click action done
-    - waiting for scheduled navigations to finish
-    - navigations have finished
-</t>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip input data pemeriksaan
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3300" yWindow="-21000" windowWidth="19200" windowHeight="19700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="22500" yWindow="-21000" windowWidth="19200" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -48,7 +48,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -448,8 +448,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:CA2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -499,6 +499,28 @@
     <col width="18.33203125" bestFit="1" customWidth="1" min="53" max="53"/>
     <col width="12.1640625" bestFit="1" customWidth="1" min="54" max="54"/>
     <col width="13.83203125" bestFit="1" customWidth="1" min="55" max="55"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="56" max="56"/>
+    <col width="17.1640625" bestFit="1" customWidth="1" style="1" min="57" max="57"/>
+    <col width="12" bestFit="1" customWidth="1" style="1" min="58" max="58"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="59" max="59"/>
+    <col width="10.5" bestFit="1" customWidth="1" style="1" min="60" max="60"/>
+    <col width="16.1640625" bestFit="1" customWidth="1" style="1" min="61" max="61"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="62" max="62"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="63" max="63"/>
+    <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="64" max="64"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="65" max="65"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="66" max="66"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="67" max="67"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="68" max="68"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="69" max="69"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="70" max="70"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="71" max="71"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="72" max="72"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="73" max="73"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="74" max="74"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="75" max="76"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="77" max="77"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="78" max="78"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -777,13 +799,128 @@
           <t>menit_olahraga_berat</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_gizi_laki</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_gula_darah</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_tensi</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_risiko_tbc</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_tbc</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_frambusia</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_kusta</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_skabies</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_telinga_mata</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_karies</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_periodontal</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_ppok</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_co</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_lipid</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_fibrosis</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_hepatitis</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_fungsi_ginjal</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_kerusakan_ginjal</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_jantung</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_kanker_usus</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_kanker_paru</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_hiv</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>periksa_sifilis</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="17" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -1026,12 +1163,127 @@
       </c>
       <c r="BD2" s="2" t="inlineStr">
         <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BJ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BK2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BL2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BM2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BN2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BO2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BP2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BQ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BR2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BS2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BT2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BU2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BV2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BW2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BX2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BY2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="BZ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
@@ -1048,6 +1300,9 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
+    <dataValidation sqref="BD2:BZ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
gula darah dewasa done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="22500" yWindow="-21000" windowWidth="19200" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28900" yWindow="-21000" windowWidth="12800" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA2"/>
+  <dimension ref="A1:CJ2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -500,27 +500,33 @@
     <col width="12.1640625" bestFit="1" customWidth="1" min="54" max="54"/>
     <col width="13.83203125" bestFit="1" customWidth="1" min="55" max="55"/>
     <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="56" max="56"/>
-    <col width="17.1640625" bestFit="1" customWidth="1" style="1" min="57" max="57"/>
-    <col width="12" bestFit="1" customWidth="1" style="1" min="58" max="58"/>
-    <col width="16" bestFit="1" customWidth="1" style="1" min="59" max="59"/>
-    <col width="10.5" bestFit="1" customWidth="1" style="1" min="60" max="60"/>
-    <col width="16.1640625" bestFit="1" customWidth="1" style="1" min="61" max="61"/>
-    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="62" max="62"/>
-    <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="63" max="63"/>
-    <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="64" max="64"/>
-    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="65" max="65"/>
-    <col width="17.5" bestFit="1" customWidth="1" style="1" min="66" max="66"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="67" max="67"/>
-    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="68" max="68"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="69" max="69"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="70" max="70"/>
-    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="71" max="71"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="72" max="72"/>
-    <col width="22" bestFit="1" customWidth="1" style="1" min="73" max="73"/>
-    <col width="14" bestFit="1" customWidth="1" style="1" min="74" max="74"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="75" max="76"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="77" max="77"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="78" max="78"/>
+    <col width="14.33203125" customWidth="1" style="1" min="57" max="59"/>
+    <col width="17.1640625" bestFit="1" customWidth="1" style="1" min="60" max="60"/>
+    <col width="14.83203125" bestFit="1" customWidth="1" style="1" min="61" max="61"/>
+    <col width="18.5" bestFit="1" customWidth="1" style="1" min="62" max="62"/>
+    <col width="18" bestFit="1" customWidth="1" style="1" min="63" max="63"/>
+    <col width="19.83203125" bestFit="1" customWidth="1" style="1" min="64" max="64"/>
+    <col width="17.1640625" customWidth="1" style="1" min="65" max="66"/>
+    <col width="12" bestFit="1" customWidth="1" style="1" min="67" max="67"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="68" max="68"/>
+    <col width="10.5" bestFit="1" customWidth="1" style="1" min="69" max="69"/>
+    <col width="16.1640625" bestFit="1" customWidth="1" style="1" min="70" max="70"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="71" max="71"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="72" max="72"/>
+    <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="73" max="73"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="74" max="74"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="75" max="75"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="76" max="76"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="77" max="77"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="78" max="78"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="79" max="79"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="80" max="80"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="81" max="81"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="82" max="82"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="83" max="83"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="84" max="85"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="86" max="86"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="87" max="87"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -806,115 +812,160 @@
       </c>
       <c r="BE1" s="1" t="inlineStr">
         <is>
+          <t>berat_badan</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>tinggi_badan</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>lingkar_perut</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
           <t>periksa_gula_darah</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>pernah_diabetes</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>total_bulan_diabetes</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>gula_darah_sewaktu</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>gula_darah_sewaktu_2</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>gula_darah_puasa</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>gula_darah_pp</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>periksa_tensi</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>periksa_risiko_tbc</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>periksa_tbc</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>periksa_frambusia</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>periksa_kusta</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>periksa_skabies</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>periksa_telinga_mata</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>periksa_karies</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>periksa_periodontal</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BX1" s="1" t="inlineStr">
         <is>
           <t>periksa_ppok</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BY1" s="1" t="inlineStr">
         <is>
           <t>periksa_co</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BZ1" s="1" t="inlineStr">
         <is>
           <t>periksa_lipid</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="CA1" s="1" t="inlineStr">
         <is>
           <t>periksa_fibrosis</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="CB1" s="1" t="inlineStr">
         <is>
           <t>periksa_hepatitis</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="CC1" s="1" t="inlineStr">
         <is>
           <t>periksa_fungsi_ginjal</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="CD1" s="1" t="inlineStr">
         <is>
           <t>periksa_kerusakan_ginjal</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="CE1" s="1" t="inlineStr">
         <is>
           <t>periksa_jantung</t>
         </is>
       </c>
-      <c r="BW1" s="1" t="inlineStr">
+      <c r="CF1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_usus</t>
         </is>
       </c>
-      <c r="BX1" s="1" t="inlineStr">
+      <c r="CG1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_paru</t>
         </is>
       </c>
-      <c r="BY1" s="1" t="inlineStr">
+      <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>periksa_hiv</t>
         </is>
       </c>
-      <c r="BZ1" s="1" t="inlineStr">
+      <c r="CI1" s="1" t="inlineStr">
         <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1168,17 +1219,17 @@
       </c>
       <c r="BE2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>80</t>
         </is>
       </c>
       <c r="BF2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>175</t>
         </is>
       </c>
       <c r="BG2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>90</t>
         </is>
       </c>
       <c r="BH2" s="2" t="inlineStr">
@@ -1188,34 +1239,26 @@
       </c>
       <c r="BI2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="BJ2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>12</t>
         </is>
       </c>
       <c r="BK2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="BL2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="BL2" s="2" t="n"/>
       <c r="BM2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="BN2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="BN2" s="2" t="n"/>
       <c r="BO2" s="2" t="inlineStr">
         <is>
           <t>True</t>
@@ -1276,7 +1319,52 @@
           <t>True</t>
         </is>
       </c>
-      <c r="CA2" t="inlineStr">
+      <c r="CA2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CB2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CC2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CD2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CE2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CF2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CG2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CH2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CI2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CJ2" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1287,7 +1375,7 @@
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -1300,7 +1388,7 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2:BZ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:CI2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
problem in do_tb -> state doesnt change
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28900" yWindow="-21000" windowWidth="12800" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18860" yWindow="9780" windowWidth="17140" windowHeight="12200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -448,8 +448,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:CX2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -509,24 +509,38 @@
     <col width="17.1640625" customWidth="1" style="1" min="65" max="66"/>
     <col width="12" bestFit="1" customWidth="1" style="1" min="67" max="67"/>
     <col width="16" bestFit="1" customWidth="1" style="1" min="68" max="68"/>
-    <col width="10.5" bestFit="1" customWidth="1" style="1" min="69" max="69"/>
-    <col width="16.1640625" bestFit="1" customWidth="1" style="1" min="70" max="70"/>
-    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="71" max="71"/>
-    <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="72" max="72"/>
-    <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="73" max="73"/>
-    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="74" max="74"/>
-    <col width="17.5" bestFit="1" customWidth="1" style="1" min="75" max="75"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="76" max="76"/>
-    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="77" max="77"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="78" max="78"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="79" max="79"/>
-    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="80" max="80"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="81" max="81"/>
-    <col width="22" bestFit="1" customWidth="1" style="1" min="82" max="82"/>
-    <col width="14" bestFit="1" customWidth="1" style="1" min="83" max="83"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="84" max="85"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="86" max="86"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="87" max="87"/>
+    <col width="19.6640625" bestFit="1" customWidth="1" style="1" min="69" max="69"/>
+    <col width="6.83203125" bestFit="1" customWidth="1" style="1" min="70" max="70"/>
+    <col width="8" bestFit="1" customWidth="1" style="1" min="71" max="71"/>
+    <col width="8.83203125" bestFit="1" customWidth="1" style="1" min="72" max="72"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="73" max="73"/>
+    <col width="16" bestFit="1" customWidth="1" style="1" min="74" max="74"/>
+    <col width="25" bestFit="1" customWidth="1" style="1" min="75" max="75"/>
+    <col width="8.33203125" bestFit="1" customWidth="1" style="1" min="76" max="76"/>
+    <col width="19.6640625" bestFit="1" customWidth="1" style="1" min="77" max="77"/>
+    <col width="17.1640625" bestFit="1" customWidth="1" style="1" min="78" max="78"/>
+    <col width="23.5" bestFit="1" customWidth="1" style="1" min="79" max="79"/>
+    <col width="14.83203125" bestFit="1" customWidth="1" style="1" min="80" max="80"/>
+    <col width="14.83203125" customWidth="1" style="1" min="81" max="81"/>
+    <col width="10.5" bestFit="1" customWidth="1" style="1" min="82" max="82"/>
+    <col width="21.33203125" bestFit="1" customWidth="1" style="1" min="83" max="83"/>
+    <col width="16.1640625" bestFit="1" customWidth="1" style="1" min="84" max="84"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="85" max="85"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="86" max="86"/>
+    <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="87" max="87"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="88" max="88"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="89" max="89"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="90" max="90"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="91" max="91"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="92" max="92"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="93" max="93"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="94" max="94"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="95" max="95"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="96" max="96"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="97" max="97"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="98" max="99"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="100" max="100"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="101" max="101"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -867,105 +881,175 @@
       </c>
       <c r="BP1" s="1" t="inlineStr">
         <is>
+          <t>pernah_hipertensi</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>total_bulan_hipertensi</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>sistolik</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>diastolik</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>sistolik_2</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>diastolik_2</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
           <t>periksa_risiko_tbc</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>pernah_batuk_tidak_sembuh</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>bb_turun</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>demam_hilang_timbul</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>berkeringat_malam</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>pembesaran_getah_bening</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>radiografi_toraks</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>hasil_rontgen</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
         <is>
           <t>periksa_tbc</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>kontak_tbc</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
         <is>
           <t>periksa_frambusia</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="CG1" s="1" t="inlineStr">
         <is>
           <t>periksa_kusta</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>periksa_skabies</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="CI1" s="1" t="inlineStr">
         <is>
           <t>periksa_telinga_mata</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="CJ1" s="1" t="inlineStr">
         <is>
           <t>periksa_karies</t>
         </is>
       </c>
-      <c r="BW1" s="1" t="inlineStr">
+      <c r="CK1" s="1" t="inlineStr">
         <is>
           <t>periksa_periodontal</t>
         </is>
       </c>
-      <c r="BX1" s="1" t="inlineStr">
+      <c r="CL1" s="1" t="inlineStr">
         <is>
           <t>periksa_ppok</t>
         </is>
       </c>
-      <c r="BY1" s="1" t="inlineStr">
+      <c r="CM1" s="1" t="inlineStr">
         <is>
           <t>periksa_co</t>
         </is>
       </c>
-      <c r="BZ1" s="1" t="inlineStr">
+      <c r="CN1" s="1" t="inlineStr">
         <is>
           <t>periksa_lipid</t>
         </is>
       </c>
-      <c r="CA1" s="1" t="inlineStr">
+      <c r="CO1" s="1" t="inlineStr">
         <is>
           <t>periksa_fibrosis</t>
         </is>
       </c>
-      <c r="CB1" s="1" t="inlineStr">
+      <c r="CP1" s="1" t="inlineStr">
         <is>
           <t>periksa_hepatitis</t>
         </is>
       </c>
-      <c r="CC1" s="1" t="inlineStr">
+      <c r="CQ1" s="1" t="inlineStr">
         <is>
           <t>periksa_fungsi_ginjal</t>
         </is>
       </c>
-      <c r="CD1" s="1" t="inlineStr">
+      <c r="CR1" s="1" t="inlineStr">
         <is>
           <t>periksa_kerusakan_ginjal</t>
         </is>
       </c>
-      <c r="CE1" s="1" t="inlineStr">
+      <c r="CS1" s="1" t="inlineStr">
         <is>
           <t>periksa_jantung</t>
         </is>
       </c>
-      <c r="CF1" s="1" t="inlineStr">
+      <c r="CT1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_usus</t>
         </is>
       </c>
-      <c r="CG1" s="1" t="inlineStr">
+      <c r="CU1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_paru</t>
         </is>
       </c>
-      <c r="CH1" s="1" t="inlineStr">
+      <c r="CV1" s="1" t="inlineStr">
         <is>
           <t>periksa_hiv</t>
         </is>
       </c>
-      <c r="CI1" s="1" t="inlineStr">
+      <c r="CW1" s="1" t="inlineStr">
         <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CX1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1266,34 +1350,26 @@
       </c>
       <c r="BP2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="BQ2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>12</t>
         </is>
       </c>
       <c r="BR2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>120</t>
         </is>
       </c>
       <c r="BS2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="BT2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="BU2" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="BT2" s="2" t="n"/>
+      <c r="BU2" s="2" t="n"/>
       <c r="BV2" s="2" t="inlineStr">
         <is>
           <t>True</t>
@@ -1301,37 +1377,37 @@
       </c>
       <c r="BW2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Tidak batuk</t>
         </is>
       </c>
       <c r="BX2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="BY2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="BZ2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="CA2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="CB2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="CC2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="CD2" s="2" t="inlineStr">
@@ -1341,7 +1417,7 @@
       </c>
       <c r="CE2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Riwayat kontak serumah</t>
         </is>
       </c>
       <c r="CF2" s="2" t="inlineStr">
@@ -1364,32 +1440,120 @@
           <t>True</t>
         </is>
       </c>
-      <c r="CJ2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
+      <c r="CJ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CK2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CL2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CM2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CN2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CO2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CP2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CQ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CR2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CS2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CU2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CV2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CW2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CX2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAILED: Locator.set_checked: Clicking the checkbox did not change its state
+Call log:
+  - waiting for locator("input#hasil-lab-1-1")
+    - locator resolved to &lt;input type="checkbox" id="hasil-lab-1-1" class="peer sr-only"/&gt;
+  - attempting click action
+    - scrolling into view if needed
+    - done scrolling
+    - forcing action
+    - performing click action
+    - click action done
+    - waiting for scheduled navigations to finish
+    - navigations have finished
+</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="9">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2 BP2 BX2:CB2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2 AE2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
+    <dataValidation sqref="J2 AE2 BW2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
     <dataValidation sqref="T2:W2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2 BH2 BN2:CI2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CF2:CW2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CE2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
still working on state change problem
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -449,7 +449,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:CX2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1512,19 +1512,7 @@
       </c>
       <c r="CX2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.set_checked: Clicking the checkbox did not change its state
-Call log:
-  - waiting for locator("input#hasil-lab-1-1")
-    - locator resolved to &lt;input type="checkbox" id="hasil-lab-1-1" class="peer sr-only"/&gt;
-  - attempting click action
-    - scrolling into view if needed
-    - done scrolling
-    - forcing action
-    - performing click action
-    - click action done
-    - waiting for scheduled navigations to finish
-    - navigations have finished
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
telinga dan mata done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF2"/>
+  <dimension ref="A1:DP2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -538,19 +538,28 @@
     <col width="14.1640625" bestFit="1" customWidth="1" style="1" min="93" max="93"/>
     <col width="14.1640625" customWidth="1" style="1" min="94" max="94"/>
     <col width="18.83203125" bestFit="1" customWidth="1" style="1" min="95" max="95"/>
-    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="96" max="96"/>
-    <col width="17.5" bestFit="1" customWidth="1" style="1" min="97" max="97"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="98" max="98"/>
-    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="99" max="99"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="100" max="100"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="101" max="101"/>
-    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="102" max="102"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="103" max="103"/>
-    <col width="22" bestFit="1" customWidth="1" style="1" min="104" max="104"/>
-    <col width="14" bestFit="1" customWidth="1" style="1" min="105" max="105"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="106" max="107"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="108" max="108"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="109" max="109"/>
+    <col width="23.6640625" bestFit="1" customWidth="1" style="1" min="96" max="96"/>
+    <col width="23.6640625" customWidth="1" style="1" min="97" max="97"/>
+    <col width="26" bestFit="1" customWidth="1" style="1" min="98" max="98"/>
+    <col width="26" customWidth="1" style="1" min="99" max="99"/>
+    <col width="36.1640625" bestFit="1" customWidth="1" style="1" min="100" max="100"/>
+    <col width="41.5" bestFit="1" customWidth="1" style="1" min="101" max="101"/>
+    <col width="29" bestFit="1" customWidth="1" style="1" min="102" max="102"/>
+    <col width="20.33203125" bestFit="1" customWidth="1" style="1" min="103" max="103"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="104" max="104"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="105" max="106"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="107" max="107"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="108" max="108"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="109" max="109"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="110" max="110"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="111" max="111"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="112" max="112"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="113" max="113"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="114" max="114"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="115" max="115"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="116" max="117"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="118" max="118"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="119" max="119"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1031,75 +1040,125 @@
       </c>
       <c r="CR1" s="1" t="inlineStr">
         <is>
+          <t>serumen_impaksi</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>infeksi_telinga</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>tajam_pendengaran</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>tes_penala</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>tajam_penglihatan</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>hasil_visus</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>pinhole</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>hasil_refraksi</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>funduskopi</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>pupil</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
           <t>periksa_karies</t>
         </is>
       </c>
-      <c r="CS1" s="1" t="inlineStr">
+      <c r="DC1" s="1" t="inlineStr">
         <is>
           <t>periksa_periodontal</t>
         </is>
       </c>
-      <c r="CT1" s="1" t="inlineStr">
+      <c r="DD1" s="1" t="inlineStr">
         <is>
           <t>periksa_ppok</t>
         </is>
       </c>
-      <c r="CU1" s="1" t="inlineStr">
+      <c r="DE1" s="1" t="inlineStr">
         <is>
           <t>periksa_co</t>
         </is>
       </c>
-      <c r="CV1" s="1" t="inlineStr">
+      <c r="DF1" s="1" t="inlineStr">
         <is>
           <t>periksa_lipid</t>
         </is>
       </c>
-      <c r="CW1" s="1" t="inlineStr">
+      <c r="DG1" s="1" t="inlineStr">
         <is>
           <t>periksa_fibrosis</t>
         </is>
       </c>
-      <c r="CX1" s="1" t="inlineStr">
+      <c r="DH1" s="1" t="inlineStr">
         <is>
           <t>periksa_hepatitis</t>
         </is>
       </c>
-      <c r="CY1" s="1" t="inlineStr">
+      <c r="DI1" s="1" t="inlineStr">
         <is>
           <t>periksa_fungsi_ginjal</t>
         </is>
       </c>
-      <c r="CZ1" s="1" t="inlineStr">
+      <c r="DJ1" s="1" t="inlineStr">
         <is>
           <t>periksa_kerusakan_ginjal</t>
         </is>
       </c>
-      <c r="DA1" s="1" t="inlineStr">
+      <c r="DK1" s="1" t="inlineStr">
         <is>
           <t>periksa_jantung</t>
         </is>
       </c>
-      <c r="DB1" s="1" t="inlineStr">
+      <c r="DL1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_usus</t>
         </is>
       </c>
-      <c r="DC1" s="1" t="inlineStr">
+      <c r="DM1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_paru</t>
         </is>
       </c>
-      <c r="DD1" s="1" t="inlineStr">
+      <c r="DN1" s="1" t="inlineStr">
         <is>
           <t>periksa_hiv</t>
         </is>
       </c>
-      <c r="DE1" s="1" t="inlineStr">
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DP1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1532,52 +1591,52 @@
       </c>
       <c r="CR2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Tidak ada serumen impaksi</t>
         </is>
       </c>
       <c r="CS2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Tidak ada infeksi telinga</t>
         </is>
       </c>
       <c r="CT2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Curiga gangguan pendengaran</t>
         </is>
       </c>
       <c r="CU2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Gangguan Pendengaran</t>
         </is>
       </c>
       <c r="CV2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Curiga gangguan penglihatan (visus &lt;6/12)</t>
         </is>
       </c>
       <c r="CW2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Gangguan penglihatan ringan (visus &lt;6/12 - 6/18)</t>
         </is>
       </c>
       <c r="CX2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Visus membaik</t>
         </is>
       </c>
       <c r="CY2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Kelainan refraksi ringan (0.50 - 3.00 Dioptri)</t>
         </is>
       </c>
       <c r="CZ2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="DA2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Curiga katarak</t>
         </is>
       </c>
       <c r="DB2" s="2" t="inlineStr">
@@ -1600,14 +1659,64 @@
           <t>True</t>
         </is>
       </c>
-      <c r="DF2" s="3" t="inlineStr">
+      <c r="DF2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DG2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DH2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DI2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DJ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DK2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DL2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DM2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DN2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DO2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DP2" s="3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="16">
+  <dataValidations count="26">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
@@ -1624,7 +1733,7 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2:DE2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2:DO2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation sqref="CC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -1653,6 +1762,36 @@
     </dataValidation>
     <dataValidation sqref="CP2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CR2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CS2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CT2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CU2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal,Gangguan Pendengaran"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CV2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CW2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CX2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CY2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="CZ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Normal,Curiga kelainan mata"</formula1>
+    </dataValidation>
+    <dataValidation sqref="DA2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
karies and periodontal done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DP2"/>
+  <dimension ref="A1:DT2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -548,18 +548,21 @@
     <col width="20.33203125" bestFit="1" customWidth="1" style="1" min="103" max="103"/>
     <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="104" max="104"/>
     <col width="12.83203125" bestFit="1" customWidth="1" style="1" min="105" max="106"/>
-    <col width="17.5" bestFit="1" customWidth="1" style="1" min="107" max="107"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="108" max="108"/>
-    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="109" max="109"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="110" max="110"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="111" max="111"/>
-    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="112" max="112"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="113" max="113"/>
-    <col width="22" bestFit="1" customWidth="1" style="1" min="114" max="114"/>
-    <col width="14" bestFit="1" customWidth="1" style="1" min="115" max="115"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="116" max="117"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="118" max="118"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="119" max="119"/>
+    <col width="12.83203125" customWidth="1" style="1" min="107" max="108"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="109" max="109"/>
+    <col width="18.5" bestFit="1" customWidth="1" style="1" min="110" max="110"/>
+    <col width="17.5" customWidth="1" style="1" min="111" max="111"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" style="1" min="112" max="112"/>
+    <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="113" max="113"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="114" max="114"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="115" max="115"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="116" max="116"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="117" max="117"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="118" max="118"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="119" max="119"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="120" max="121"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="122" max="122"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="123" max="123"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,70 +1098,90 @@
       </c>
       <c r="DC1" s="1" t="inlineStr">
         <is>
+          <t>gigi_karies</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>gigi_hilang</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
           <t>periksa_periodontal</t>
         </is>
       </c>
-      <c r="DD1" s="1" t="inlineStr">
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>penyakit_periodontal</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>gigi_goyang</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
         <is>
           <t>periksa_ppok</t>
         </is>
       </c>
-      <c r="DE1" s="1" t="inlineStr">
+      <c r="DI1" s="1" t="inlineStr">
         <is>
           <t>periksa_co</t>
         </is>
       </c>
-      <c r="DF1" s="1" t="inlineStr">
+      <c r="DJ1" s="1" t="inlineStr">
         <is>
           <t>periksa_lipid</t>
         </is>
       </c>
-      <c r="DG1" s="1" t="inlineStr">
+      <c r="DK1" s="1" t="inlineStr">
         <is>
           <t>periksa_fibrosis</t>
         </is>
       </c>
-      <c r="DH1" s="1" t="inlineStr">
+      <c r="DL1" s="1" t="inlineStr">
         <is>
           <t>periksa_hepatitis</t>
         </is>
       </c>
-      <c r="DI1" s="1" t="inlineStr">
+      <c r="DM1" s="1" t="inlineStr">
         <is>
           <t>periksa_fungsi_ginjal</t>
         </is>
       </c>
-      <c r="DJ1" s="1" t="inlineStr">
+      <c r="DN1" s="1" t="inlineStr">
         <is>
           <t>periksa_kerusakan_ginjal</t>
         </is>
       </c>
-      <c r="DK1" s="1" t="inlineStr">
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>periksa_jantung</t>
         </is>
       </c>
-      <c r="DL1" s="1" t="inlineStr">
+      <c r="DP1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_usus</t>
         </is>
       </c>
-      <c r="DM1" s="1" t="inlineStr">
+      <c r="DQ1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_paru</t>
         </is>
       </c>
-      <c r="DN1" s="1" t="inlineStr">
+      <c r="DR1" s="1" t="inlineStr">
         <is>
           <t>periksa_hiv</t>
         </is>
       </c>
-      <c r="DO1" s="1" t="inlineStr">
+      <c r="DS1" s="1" t="inlineStr">
         <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="DP1" t="inlineStr">
+      <c r="DT1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1646,12 +1669,12 @@
       </c>
       <c r="DC2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="DD2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Tidak</t>
         </is>
       </c>
       <c r="DE2" s="2" t="inlineStr">
@@ -1661,12 +1684,12 @@
       </c>
       <c r="DF2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="DG2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="DH2" s="2" t="inlineStr">
@@ -1709,7 +1732,27 @@
           <t>True</t>
         </is>
       </c>
-      <c r="DP2" s="3" t="inlineStr">
+      <c r="DP2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DQ2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DR2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DS2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="DT2" s="3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -1720,7 +1763,7 @@
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2 BP2 BX2:CB2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2 BP2 BX2:CB2 DC2 DD2 DF2:DG2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -1733,7 +1776,7 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2:DO2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2:DS2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation sqref="CC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">

</xml_diff>

<commit_message>
lipid fibrosis hepatitis done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ2"/>
+  <dimension ref="A1:EJ2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -558,15 +558,22 @@
     <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="115" max="115"/>
     <col width="19.5" customWidth="1" style="1" min="116" max="118"/>
     <col width="9.83203125" bestFit="1" customWidth="1" style="1" min="119" max="119"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="120" max="120"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="121" max="121"/>
-    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="122" max="122"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="123" max="123"/>
-    <col width="22" bestFit="1" customWidth="1" style="1" min="124" max="124"/>
-    <col width="14" bestFit="1" customWidth="1" style="1" min="125" max="125"/>
-    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="126" max="127"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="128" max="128"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="129" max="129"/>
+    <col width="9.83203125" customWidth="1" style="1" min="120" max="120"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="121" max="121"/>
+    <col width="11.5" customWidth="1" style="1" min="122" max="125"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" style="1" min="126" max="126"/>
+    <col width="4.5" bestFit="1" customWidth="1" style="1" min="127" max="127"/>
+    <col width="9" bestFit="1" customWidth="1" style="1" min="128" max="128"/>
+    <col width="15.1640625" bestFit="1" customWidth="1" style="1" min="129" max="129"/>
+    <col width="15.1640625" customWidth="1" style="1" min="130" max="130"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="131" max="131"/>
+    <col width="18.1640625" customWidth="1" style="1" min="132" max="132"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="133" max="133"/>
+    <col width="22" bestFit="1" customWidth="1" style="1" min="134" max="134"/>
+    <col width="14" bestFit="1" customWidth="1" style="1" min="135" max="135"/>
+    <col width="18.1640625" bestFit="1" customWidth="1" style="1" min="136" max="137"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="138" max="138"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="139" max="139"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1167,55 +1174,105 @@
       </c>
       <c r="DP1" s="1" t="inlineStr">
         <is>
+          <t>kadar_co</t>
+        </is>
+      </c>
+      <c r="DQ1" s="1" t="inlineStr">
+        <is>
           <t>periksa_lipid</t>
         </is>
       </c>
-      <c r="DQ1" s="1" t="inlineStr">
+      <c r="DR1" s="1" t="inlineStr">
+        <is>
+          <t>kolesterol</t>
+        </is>
+      </c>
+      <c r="DS1" s="1" t="inlineStr">
+        <is>
+          <t>hdl</t>
+        </is>
+      </c>
+      <c r="DT1" s="1" t="inlineStr">
+        <is>
+          <t>ldl</t>
+        </is>
+      </c>
+      <c r="DU1" s="1" t="inlineStr">
+        <is>
+          <t>trigliserida</t>
+        </is>
+      </c>
+      <c r="DV1" s="1" t="inlineStr">
         <is>
           <t>periksa_fibrosis</t>
         </is>
       </c>
-      <c r="DR1" s="1" t="inlineStr">
+      <c r="DW1" s="1" t="inlineStr">
+        <is>
+          <t>sgot</t>
+        </is>
+      </c>
+      <c r="DX1" s="1" t="inlineStr">
+        <is>
+          <t>trombosit</t>
+        </is>
+      </c>
+      <c r="DY1" s="1" t="inlineStr">
         <is>
           <t>periksa_hepatitis</t>
         </is>
       </c>
-      <c r="DS1" s="1" t="inlineStr">
+      <c r="DZ1" s="1" t="inlineStr">
+        <is>
+          <t>hepatitis_b</t>
+        </is>
+      </c>
+      <c r="EA1" s="1" t="inlineStr">
+        <is>
+          <t>hepatitis_c</t>
+        </is>
+      </c>
+      <c r="EB1" s="1" t="inlineStr">
+        <is>
+          <t>vl_hepatitis_c</t>
+        </is>
+      </c>
+      <c r="EC1" s="1" t="inlineStr">
         <is>
           <t>periksa_fungsi_ginjal</t>
         </is>
       </c>
-      <c r="DT1" s="1" t="inlineStr">
+      <c r="ED1" s="1" t="inlineStr">
         <is>
           <t>periksa_kerusakan_ginjal</t>
         </is>
       </c>
-      <c r="DU1" s="1" t="inlineStr">
+      <c r="EE1" s="1" t="inlineStr">
         <is>
           <t>periksa_jantung</t>
         </is>
       </c>
-      <c r="DV1" s="1" t="inlineStr">
+      <c r="EF1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_usus</t>
         </is>
       </c>
-      <c r="DW1" s="1" t="inlineStr">
+      <c r="EG1" s="1" t="inlineStr">
         <is>
           <t>periksa_kanker_paru</t>
         </is>
       </c>
-      <c r="DX1" s="1" t="inlineStr">
+      <c r="EH1" s="1" t="inlineStr">
         <is>
           <t>periksa_hiv</t>
         </is>
       </c>
-      <c r="DY1" s="1" t="inlineStr">
+      <c r="EI1" s="1" t="inlineStr">
         <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="DZ1" t="inlineStr">
+      <c r="EJ1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1768,7 +1825,7 @@
       </c>
       <c r="DP2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>90</t>
         </is>
       </c>
       <c r="DQ2" s="2" t="inlineStr">
@@ -1778,22 +1835,22 @@
       </c>
       <c r="DR2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>200</t>
         </is>
       </c>
       <c r="DS2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>200</t>
         </is>
       </c>
       <c r="DT2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>240</t>
         </is>
       </c>
       <c r="DU2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>100</t>
         </is>
       </c>
       <c r="DV2" s="2" t="inlineStr">
@@ -1803,12 +1860,12 @@
       </c>
       <c r="DW2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>45</t>
         </is>
       </c>
       <c r="DX2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>22</t>
         </is>
       </c>
       <c r="DY2" s="2" t="inlineStr">
@@ -1816,14 +1873,64 @@
           <t>True</t>
         </is>
       </c>
-      <c r="DZ2" s="3" t="inlineStr">
+      <c r="DZ2" s="2" t="inlineStr">
+        <is>
+          <t>HBsAg Non Reaktif</t>
+        </is>
+      </c>
+      <c r="EA2" s="2" t="inlineStr">
+        <is>
+          <t>Anti HCV Reaktif</t>
+        </is>
+      </c>
+      <c r="EB2" s="2" t="inlineStr">
+        <is>
+          <t>VL HCV RNA Negatif</t>
+        </is>
+      </c>
+      <c r="EC2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="ED2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EE2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EF2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EG2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EH2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EI2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="EJ2" s="3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="28">
+  <dataValidations count="31">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
@@ -1840,7 +1947,7 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2:DY2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2 DQ2 DV2 DY2 EC2:EI2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation sqref="CC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -1905,6 +2012,15 @@
     </dataValidation>
     <dataValidation sqref="DJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
+    </dataValidation>
+    <dataValidation sqref="DZ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
+    </dataValidation>
+    <dataValidation sqref="EA2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
+    </dataValidation>
+    <dataValidation sqref="EB2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
hiv and sifilis done
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FC2"/>
+  <dimension ref="A1:FH2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -588,7 +588,9 @@
     <col width="43.1640625" bestFit="1" customWidth="1" style="1" min="154" max="154"/>
     <col width="18.1640625" customWidth="1" style="1" min="155" max="156"/>
     <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="157" max="157"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="158" max="158"/>
+    <col width="10.33203125" customWidth="1" style="1" min="158" max="161"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" style="1" min="162" max="162"/>
+    <col width="12.1640625" customWidth="1" style="1" min="163" max="163"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1379,10 +1381,35 @@
       </c>
       <c r="FB1" s="1" t="inlineStr">
         <is>
+          <t>rapid_test</t>
+        </is>
+      </c>
+      <c r="FC1" s="1" t="inlineStr">
+        <is>
+          <t>r2_hiv</t>
+        </is>
+      </c>
+      <c r="FD1" s="1" t="inlineStr">
+        <is>
+          <t>r1_hiv_ulang</t>
+        </is>
+      </c>
+      <c r="FE1" s="1" t="inlineStr">
+        <is>
+          <t>r3_hiv</t>
+        </is>
+      </c>
+      <c r="FF1" s="1" t="inlineStr">
+        <is>
           <t>periksa_sifilis</t>
         </is>
       </c>
-      <c r="FC1" t="inlineStr">
+      <c r="FG1" s="1" t="inlineStr">
+        <is>
+          <t>rapid_test_sifilis</t>
+        </is>
+      </c>
+      <c r="FH1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -2125,10 +2152,35 @@
       </c>
       <c r="FB2" s="2" t="inlineStr">
         <is>
+          <t>Reaktif</t>
+        </is>
+      </c>
+      <c r="FC2" s="2" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="FD2" s="2" t="inlineStr">
+        <is>
+          <t>Non Reaktif</t>
+        </is>
+      </c>
+      <c r="FE2" s="2" t="inlineStr">
+        <is>
+          <t>Reaktif</t>
+        </is>
+      </c>
+      <c r="FF2" s="2" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="FC2" s="3" t="inlineStr">
+      <c r="FG2" s="2" t="inlineStr">
+        <is>
+          <t>Reaktif</t>
+        </is>
+      </c>
+      <c r="FH2" s="3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
@@ -2152,7 +2204,7 @@
     <dataValidation sqref="AJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2 DQ2 DV2 DY2 EC2 EH2 EK2 EN2 ER2 FA2:FB2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="BD2 BH2 BN2:BO2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2 DQ2 DV2 DY2 EC2 EH2 EK2 EN2 ER2 FA2 FF2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation sqref="CC2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -2170,7 +2222,7 @@
     <dataValidation sqref="CJ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation sqref="CK2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="CK2 FB2:FE2 FG2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
     <dataValidation sqref="CM2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">

</xml_diff>

<commit_message>
patching on excel file and comment
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="24560" yWindow="-13380" windowWidth="17140" windowHeight="12200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3300" yWindow="-21000" windowWidth="38400" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,12 +16,31 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -128,6 +147,247 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Microsoft Office User</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi jika status_perkawinan selain Menikah</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila merokok_setahun_terakhir adalah Ya</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila merokok_setahun_terakhir_b nilainya Ya</t>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila merokok_setahun_terakhir_b nilainya Ya
+</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila merokok_setahun_terakhir_b nilainya Ya
+</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila merokok_setahun_terakhir_b nilainya Tidak</t>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+Wajib diisi apabila pernah_merokok nilainya Ya</t>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+Wajib diisi apabila pernah_merokok nilainya Ya
+</t>
+      </text>
+    </comment>
+    <comment ref="AM1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila aktivitas_domestik Ya</t>
+      </text>
+    </comment>
+    <comment ref="AN1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_domestik Ya </t>
+      </text>
+    </comment>
+    <comment ref="AP1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_pekerjaan Ya </t>
+      </text>
+    </comment>
+    <comment ref="AQ1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_pekerjaan Ya </t>
+      </text>
+    </comment>
+    <comment ref="AS1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_perjalanan Ya </t>
+      </text>
+    </comment>
+    <comment ref="AT1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_perjalanan Ya </t>
+      </text>
+    </comment>
+    <comment ref="AV1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_olahraga Ya </t>
+      </text>
+    </comment>
+    <comment ref="AW1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_olahraga Ya </t>
+      </text>
+    </comment>
+    <comment ref="AY1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_kerja_berat Ya </t>
+      </text>
+    </comment>
+    <comment ref="AZ1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_kerja_berat Ya </t>
+      </text>
+    </comment>
+    <comment ref="BB1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_olahraga_berat Ya </t>
+      </text>
+    </comment>
+    <comment ref="BC1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila aktivitas_olahraga_berat Ya </t>
+      </text>
+    </comment>
+    <comment ref="BJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila pernah_diabetes Ya</t>
+      </text>
+    </comment>
+    <comment ref="BK1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Microsoft Office User:
+wajib diisi apabila pernah_diabetes Ya </t>
+      </text>
+    </comment>
+    <comment ref="BL1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila pernah_diabetes Tidak</t>
+      </text>
+    </comment>
+    <comment ref="BQ1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila pernah_hipertensi Ya</t>
+      </text>
+    </comment>
+    <comment ref="CC1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila radiografi_toraks Ya</t>
+      </text>
+    </comment>
+    <comment ref="CF1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila riwayat kontak serumah atau riwayat kontak erat</t>
+      </text>
+    </comment>
+    <comment ref="CK1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila Suspek Frambusia</t>
+      </text>
+    </comment>
+    <comment ref="CN1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila bercak_putih Meragukan</t>
+      </text>
+    </comment>
+    <comment ref="CU1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila Curiga gangguan pendengaran</t>
+      </text>
+    </comment>
+    <comment ref="CW1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila Curiga gangguan penglihatan</t>
+      </text>
+    </comment>
+    <comment ref="CX1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila hasil visus selain Normal</t>
+      </text>
+    </comment>
+    <comment ref="CY1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila pinhole Visus membaik</t>
+      </text>
+    </comment>
+    <comment ref="CZ1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila pinhole bukan Visus membaik</t>
+      </text>
+    </comment>
+    <comment ref="DJ1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila ppok_merokok Iya</t>
+      </text>
+    </comment>
+    <comment ref="EB1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila hepatitis_c Anti HCV Reaktif</t>
+      </text>
+    </comment>
+    <comment ref="FC1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila rapid_test Reaktif</t>
+      </text>
+    </comment>
+    <comment ref="FD1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila r2_hiv Non Reaktif</t>
+      </text>
+    </comment>
+    <comment ref="FE1" authorId="0" shapeId="0">
+      <text>
+        <t>Microsoft Office User:
+wajib diisi apabila r2_hiv Reaktif</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -458,7 +718,7 @@
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
     <col width="11.5" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
     <col width="10.5" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="16.6640625" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="14.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="10.83203125" customWidth="1" style="1" min="7" max="7"/>
     <col width="8.1640625" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
@@ -2187,17 +2447,17 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="44">
+  <dataValidations disablePrompts="1" count="42">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2 BP2 BX2:CB2 DC2 DD2 DF2:DG2 DK2:DN2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2 H2:I2 K2:S2 X2:AD2 AH2 AK2:AL2 AO2 AR2 AU2 AX2 BA2 BI2 BP2 BX2:CB2 DC2:DD2 DF2:DG2 DK2:DN2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation sqref="G2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2 AE2 BW2 CH2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
+    <dataValidation sqref="J2 AE2 BW2 CH2 EV2 EY2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
     <dataValidation sqref="T2:W2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
@@ -2303,19 +2563,18 @@
     <dataValidation sqref="EU2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation sqref="EV2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
     <dataValidation sqref="EW2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
     <dataValidation sqref="EX2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation sqref="EY2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list"/>
     <dataValidation sqref="EZ2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
wip kanker leher rahim
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACB9594-7C8A-2C42-8567-B1B96047AEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E43E2EC-1E8E-7343-ACD4-81C41161473F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3300" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -88,7 +88,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -103,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -119,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="AI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -135,7 +135,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -150,7 +150,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="AK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -165,7 +165,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -181,7 +181,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -196,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="AP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -211,7 +211,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="AR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -226,7 +226,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="AS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -241,7 +241,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -256,7 +256,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -271,7 +271,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="AX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -286,7 +286,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
+    <comment ref="AY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
       <text>
         <r>
           <rPr>
@@ -301,7 +301,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
       <text>
         <r>
           <rPr>
@@ -316,7 +316,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
+    <comment ref="BB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
       <text>
         <r>
           <rPr>
@@ -331,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
+    <comment ref="BD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
       <text>
         <r>
           <rPr>
@@ -346,7 +346,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
+    <comment ref="BE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
       <text>
         <r>
           <rPr>
@@ -361,7 +361,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
+    <comment ref="BL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
       <text>
         <r>
           <rPr>
@@ -376,7 +376,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
+    <comment ref="BM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
       <text>
         <r>
           <rPr>
@@ -391,7 +391,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
+    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
       <text>
         <r>
           <rPr>
@@ -406,7 +406,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
+    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
       <text>
         <r>
           <rPr>
@@ -421,7 +421,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
+    <comment ref="CE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
       <text>
         <r>
           <rPr>
@@ -436,7 +436,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
+    <comment ref="CH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
       <text>
         <r>
           <rPr>
@@ -451,7 +451,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
+    <comment ref="CM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
       <text>
         <r>
           <rPr>
@@ -466,7 +466,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
+    <comment ref="CP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
       <text>
         <r>
           <rPr>
@@ -481,7 +481,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
+    <comment ref="CW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
       <text>
         <r>
           <rPr>
@@ -496,7 +496,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
+    <comment ref="CY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
       <text>
         <r>
           <rPr>
@@ -511,7 +511,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
+    <comment ref="CZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
       <text>
         <r>
           <rPr>
@@ -526,7 +526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
+    <comment ref="DA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
       <text>
         <r>
           <rPr>
@@ -541,7 +541,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
+    <comment ref="DB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
       <text>
         <r>
           <rPr>
@@ -556,7 +556,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
+    <comment ref="DL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
       <text>
         <r>
           <rPr>
@@ -571,7 +571,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
+    <comment ref="ED1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
       <text>
         <r>
           <rPr>
@@ -586,7 +586,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
+    <comment ref="FE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
       <text>
         <r>
           <rPr>
@@ -601,7 +601,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000025000000}">
+    <comment ref="FF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000025000000}">
       <text>
         <r>
           <rPr>
@@ -616,7 +616,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000026000000}">
+    <comment ref="FG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000026000000}">
       <text>
         <r>
           <rPr>
@@ -636,7 +636,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="229">
   <si>
     <t>batas_awal</t>
   </si>
@@ -1320,6 +1320,9 @@
   </si>
   <si>
     <t>sedang_hamil</t>
+  </si>
+  <si>
+    <t>pernah_seks</t>
   </si>
 </sst>
 </file>
@@ -1711,7 +1714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FI2"/>
+  <dimension ref="A1:FJ2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1731,130 +1734,131 @@
     <col min="16" max="16" width="11.5" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16.5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17" bestFit="1" customWidth="1"/>
-    <col min="22" max="24" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="49" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="23" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="16" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="16" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="58" max="60" width="14.33203125" style="1" customWidth="1"/>
-    <col min="61" max="61" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="18.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="17.1640625" style="1" customWidth="1"/>
-    <col min="68" max="68" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="23.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="14.83203125" style="1" customWidth="1"/>
-    <col min="83" max="83" width="10.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="22.83203125" style="1" customWidth="1"/>
-    <col min="88" max="88" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="16.1640625" style="1" customWidth="1"/>
-    <col min="90" max="90" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="92" max="93" width="12.33203125" style="1" customWidth="1"/>
-    <col min="94" max="94" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="14.1640625" style="1" customWidth="1"/>
-    <col min="96" max="96" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="23.6640625" style="1" customWidth="1"/>
-    <col min="99" max="99" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="26" style="1" customWidth="1"/>
-    <col min="101" max="101" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="41.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="106" max="107" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="108" max="109" width="12.83203125" style="1" customWidth="1"/>
-    <col min="110" max="110" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="18.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="17.5" style="1" customWidth="1"/>
-    <col min="113" max="113" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="19.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="117" max="119" width="19.5" style="1" customWidth="1"/>
-    <col min="120" max="120" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="9.83203125" style="1" customWidth="1"/>
-    <col min="122" max="122" width="11.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="123" max="126" width="11.5" style="1" customWidth="1"/>
-    <col min="127" max="127" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="4.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="18.1640625" style="1" customWidth="1"/>
-    <col min="134" max="134" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="136" max="138" width="8.33203125" style="1" customWidth="1"/>
-    <col min="139" max="139" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="140" max="140" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="141" max="141" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="143" max="143" width="14" style="1" customWidth="1"/>
-    <col min="144" max="144" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="18.1640625" style="1" customWidth="1"/>
-    <col min="147" max="147" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="149" max="149" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="150" max="152" width="18.1640625" style="1" customWidth="1"/>
-    <col min="153" max="153" width="46.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="154" max="154" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="155" max="155" width="43.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="156" max="157" width="18.1640625" style="1" customWidth="1"/>
-    <col min="158" max="158" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="159" max="162" width="10.33203125" style="1" customWidth="1"/>
-    <col min="163" max="163" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="12.1640625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5" customWidth="1"/>
+    <col min="22" max="22" width="17" bestFit="1" customWidth="1"/>
+    <col min="23" max="25" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="49" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="23" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="16" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="16" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="59" max="61" width="14.33203125" style="1" customWidth="1"/>
+    <col min="62" max="62" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="18.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="67" max="68" width="17.1640625" style="1" customWidth="1"/>
+    <col min="69" max="69" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="25" style="1" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="14.83203125" style="1" customWidth="1"/>
+    <col min="84" max="84" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="22.83203125" style="1" customWidth="1"/>
+    <col min="89" max="89" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="16.1640625" style="1" customWidth="1"/>
+    <col min="91" max="91" width="19.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="93" max="94" width="12.33203125" style="1" customWidth="1"/>
+    <col min="95" max="95" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="14.1640625" style="1" customWidth="1"/>
+    <col min="97" max="97" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="23.6640625" style="1" customWidth="1"/>
+    <col min="100" max="100" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="26" style="1" customWidth="1"/>
+    <col min="102" max="102" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="41.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="107" max="108" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="109" max="110" width="12.83203125" style="1" customWidth="1"/>
+    <col min="111" max="111" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="18.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="17.5" style="1" customWidth="1"/>
+    <col min="114" max="114" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="19.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="118" max="120" width="19.5" style="1" customWidth="1"/>
+    <col min="121" max="121" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="9.83203125" style="1" customWidth="1"/>
+    <col min="123" max="123" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="124" max="127" width="11.5" style="1" customWidth="1"/>
+    <col min="128" max="128" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="4.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="18.1640625" style="1" customWidth="1"/>
+    <col min="135" max="135" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="136" max="136" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="137" max="139" width="8.33203125" style="1" customWidth="1"/>
+    <col min="140" max="140" width="22" style="1" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="143" max="143" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="144" max="144" width="14" style="1" customWidth="1"/>
+    <col min="145" max="145" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="147" max="147" width="18.1640625" style="1" customWidth="1"/>
+    <col min="148" max="148" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="149" max="149" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="150" max="150" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="151" max="153" width="18.1640625" style="1" customWidth="1"/>
+    <col min="154" max="154" width="46.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="155" max="155" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="156" max="156" width="43.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="157" max="158" width="18.1640625" style="1" customWidth="1"/>
+    <col min="159" max="159" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="160" max="163" width="10.33203125" style="1" customWidth="1"/>
+    <col min="164" max="164" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="12.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:165" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:166" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1916,442 +1920,445 @@
         <v>18</v>
       </c>
       <c r="U1" t="s">
+        <v>228</v>
+      </c>
+      <c r="V1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>46</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>47</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>48</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>49</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>50</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>51</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>53</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>54</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CB1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CC1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="CE1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="CE1" s="1" t="s">
+      <c r="CF1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="CF1" s="1" t="s">
+      <c r="CG1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="CG1" s="1" t="s">
+      <c r="CH1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="CH1" s="1" t="s">
+      <c r="CI1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="CI1" s="1" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="CK1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="CL1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="CL1" s="1" t="s">
+      <c r="CM1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="CM1" s="1" t="s">
+      <c r="CN1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="CN1" s="1" t="s">
+      <c r="CO1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="CO1" s="1" t="s">
+      <c r="CP1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="CP1" s="1" t="s">
+      <c r="CQ1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="CQ1" s="1" t="s">
+      <c r="CR1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="CS1" s="1" t="s">
+      <c r="CT1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="CT1" s="1" t="s">
+      <c r="CU1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="CU1" s="1" t="s">
+      <c r="CV1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="CV1" s="1" t="s">
+      <c r="CW1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="CW1" s="1" t="s">
+      <c r="CX1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="CX1" s="1" t="s">
+      <c r="CY1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="CY1" s="1" t="s">
+      <c r="CZ1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="CZ1" s="1" t="s">
+      <c r="DA1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="DA1" s="1" t="s">
+      <c r="DB1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="DB1" s="1" t="s">
+      <c r="DC1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="DC1" s="1" t="s">
+      <c r="DD1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="DD1" s="1" t="s">
+      <c r="DE1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="DE1" s="1" t="s">
+      <c r="DF1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="DF1" s="1" t="s">
+      <c r="DG1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="DG1" s="1" t="s">
+      <c r="DH1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="DH1" s="1" t="s">
+      <c r="DI1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="DI1" s="1" t="s">
+      <c r="DJ1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="DJ1" s="1" t="s">
+      <c r="DK1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="DK1" s="1" t="s">
+      <c r="DL1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="DL1" s="1" t="s">
+      <c r="DM1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="DM1" s="1" t="s">
+      <c r="DN1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="DN1" s="1" t="s">
+      <c r="DO1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="DO1" s="1" t="s">
+      <c r="DP1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="DP1" s="1" t="s">
+      <c r="DQ1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="DQ1" s="1" t="s">
+      <c r="DR1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="DR1" s="1" t="s">
+      <c r="DS1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="DS1" s="1" t="s">
+      <c r="DT1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="DT1" s="1" t="s">
+      <c r="DU1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="DU1" s="1" t="s">
+      <c r="DV1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="DV1" s="1" t="s">
+      <c r="DW1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="DW1" s="1" t="s">
+      <c r="DX1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="DX1" s="1" t="s">
+      <c r="DY1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="DY1" s="1" t="s">
+      <c r="DZ1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="DZ1" s="1" t="s">
+      <c r="EA1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="EA1" s="1" t="s">
+      <c r="EB1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="EF1" s="1" t="s">
+      <c r="EG1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="EG1" s="1" t="s">
+      <c r="EH1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="EH1" s="1" t="s">
+      <c r="EI1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="EI1" s="1" t="s">
+      <c r="EJ1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="EJ1" s="1" t="s">
+      <c r="EK1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="EK1" s="1" t="s">
+      <c r="EL1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="EL1" s="1" t="s">
+      <c r="EM1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="EM1" s="1" t="s">
+      <c r="EN1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="EN1" s="1" t="s">
+      <c r="EO1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="EO1" s="1" t="s">
+      <c r="EP1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="EP1" s="1" t="s">
+      <c r="EQ1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="EQ1" s="1" t="s">
+      <c r="ER1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="ER1" s="1" t="s">
+      <c r="ES1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="ES1" s="1" t="s">
+      <c r="ET1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="ET1" s="1" t="s">
+      <c r="EU1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="EU1" s="1" t="s">
+      <c r="EV1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="EV1" s="1" t="s">
+      <c r="EW1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="EW1" s="1" t="s">
+      <c r="EX1" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="EX1" s="1" t="s">
+      <c r="EY1" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="EY1" s="1" t="s">
+      <c r="EZ1" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="EZ1" s="1" t="s">
+      <c r="FA1" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="FA1" s="1" t="s">
+      <c r="FB1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="FB1" s="1" t="s">
+      <c r="FC1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="FC1" s="1" t="s">
+      <c r="FD1" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="FD1" s="1" t="s">
+      <c r="FE1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="FE1" s="1" t="s">
+      <c r="FF1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="FF1" s="1" t="s">
+      <c r="FG1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="FG1" s="1" t="s">
+      <c r="FH1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="FH1" s="1" t="s">
+      <c r="FI1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="FI1" t="s">
+      <c r="FJ1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:165" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:166" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>164</v>
       </c>
@@ -2367,7 +2374,9 @@
       <c r="F2" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>168</v>
+      </c>
       <c r="H2" s="1" t="s">
         <v>169</v>
       </c>
@@ -2408,7 +2417,7 @@
         <v>168</v>
       </c>
       <c r="U2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="V2" t="s">
         <v>172</v>
@@ -2420,10 +2429,10 @@
         <v>172</v>
       </c>
       <c r="Y2" t="s">
+        <v>172</v>
+      </c>
+      <c r="Z2" t="s">
         <v>170</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>168</v>
       </c>
       <c r="AA2" t="s">
         <v>168</v>
@@ -2438,137 +2447,137 @@
         <v>168</v>
       </c>
       <c r="AE2" t="s">
+        <v>168</v>
+      </c>
+      <c r="AF2" t="s">
         <v>170</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>173</v>
       </c>
-      <c r="AG2">
+      <c r="AH2">
         <v>3</v>
       </c>
-      <c r="AH2">
+      <c r="AI2">
         <v>15</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AJ2" t="s">
         <v>170</v>
       </c>
-      <c r="AJ2">
+      <c r="AK2">
         <v>3</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AL2" t="s">
         <v>174</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>170</v>
       </c>
       <c r="AM2" t="s">
         <v>170</v>
       </c>
-      <c r="AN2">
+      <c r="AN2" t="s">
+        <v>170</v>
+      </c>
+      <c r="AO2">
         <v>5</v>
       </c>
-      <c r="AO2">
+      <c r="AP2">
         <v>60</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AQ2" t="s">
         <v>170</v>
       </c>
-      <c r="AQ2">
+      <c r="AR2">
         <v>6</v>
       </c>
-      <c r="AR2">
+      <c r="AS2">
         <v>30</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>170</v>
       </c>
-      <c r="AT2">
+      <c r="AU2">
         <v>3</v>
       </c>
-      <c r="AU2">
+      <c r="AV2">
         <v>120</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>170</v>
       </c>
-      <c r="AW2">
+      <c r="AX2">
         <v>2</v>
       </c>
-      <c r="AX2">
+      <c r="AY2">
         <v>100</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AZ2" t="s">
         <v>170</v>
       </c>
-      <c r="AZ2">
+      <c r="BA2">
         <v>1</v>
       </c>
-      <c r="BA2">
+      <c r="BB2">
         <v>20</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BC2" t="s">
         <v>170</v>
       </c>
-      <c r="BC2">
+      <c r="BD2">
         <v>1</v>
       </c>
-      <c r="BD2">
+      <c r="BE2">
         <v>20</v>
       </c>
-      <c r="BE2" s="2" t="s">
+      <c r="BF2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="BF2" s="2" t="s">
+      <c r="BG2" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="BG2" s="2" t="s">
+      <c r="BH2" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="BH2" s="2" t="s">
+      <c r="BI2" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="BI2" s="2" t="s">
+      <c r="BJ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="BJ2" s="2" t="s">
+      <c r="BK2" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="BK2" s="2" t="s">
+      <c r="BL2" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="BL2" s="2" t="s">
+      <c r="BM2" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="BM2" s="2"/>
-      <c r="BN2" s="2" t="s">
+      <c r="BN2" s="2"/>
+      <c r="BO2" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="BO2" s="2"/>
-      <c r="BP2" s="2" t="s">
+      <c r="BP2" s="2"/>
+      <c r="BQ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="BQ2" s="2" t="s">
+      <c r="BR2" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="BR2" s="2" t="s">
+      <c r="BS2" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="BS2" s="2" t="s">
+      <c r="BT2" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="BT2" s="2" t="s">
+      <c r="BU2" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="BU2" s="2"/>
       <c r="BV2" s="2"/>
-      <c r="BW2" s="2" t="s">
+      <c r="BW2" s="2"/>
+      <c r="BX2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="BX2" s="2" t="s">
+      <c r="BY2" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="BY2" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="BZ2" s="2" t="s">
         <v>170</v>
@@ -2583,109 +2592,109 @@
         <v>170</v>
       </c>
       <c r="CD2" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="CE2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="CE2" s="2" t="s">
+      <c r="CF2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="CF2" s="2" t="s">
+      <c r="CG2" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="CG2" s="2" t="s">
+      <c r="CH2" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="CH2" s="2" t="s">
+      <c r="CI2" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="CI2" s="2" t="s">
+      <c r="CJ2" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="CJ2" s="2" t="s">
+      <c r="CK2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="CK2" s="2" t="s">
+      <c r="CL2" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="CL2" s="2" t="s">
+      <c r="CM2" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="CM2" s="2" t="s">
+      <c r="CN2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="CN2" s="2" t="s">
+      <c r="CO2" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="CO2" s="2" t="s">
+      <c r="CP2" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="CP2" s="2" t="s">
+      <c r="CQ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="CQ2" s="2" t="s">
+      <c r="CR2" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="CR2" s="2" t="s">
+      <c r="CS2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="CS2" s="2" t="s">
+      <c r="CT2" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="CT2" s="2" t="s">
+      <c r="CU2" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="CU2" s="2" t="s">
+      <c r="CV2" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="CV2" s="2" t="s">
+      <c r="CW2" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="CW2" s="2" t="s">
+      <c r="CX2" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="CX2" s="2" t="s">
+      <c r="CY2" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="CY2" s="2" t="s">
+      <c r="CZ2" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="CZ2" s="2" t="s">
+      <c r="DA2" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="DA2" s="2" t="s">
+      <c r="DB2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="DB2" s="2" t="s">
+      <c r="DC2" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="DC2" s="2" t="s">
+      <c r="DD2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="DD2" s="2" t="s">
+      <c r="DE2" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="DE2" s="2" t="s">
+      <c r="DF2" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="DF2" s="2" t="s">
+      <c r="DG2" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="DG2" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="DH2" s="2" t="s">
         <v>170</v>
       </c>
       <c r="DI2" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="DJ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="DJ2" s="2" t="s">
+      <c r="DK2" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="DK2" s="2" t="s">
+      <c r="DL2" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="DL2" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="DM2" s="2" t="s">
         <v>170</v>
@@ -2697,266 +2706,269 @@
         <v>170</v>
       </c>
       <c r="DP2" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="DQ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="DQ2" s="2" t="s">
+      <c r="DR2" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="DR2" s="2" t="s">
+      <c r="DS2" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="DS2" s="2" t="s">
-        <v>204</v>
       </c>
       <c r="DT2" s="2" t="s">
         <v>204</v>
       </c>
       <c r="DU2" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="DV2" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="DV2" s="2" t="s">
+      <c r="DW2" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="DW2" s="2" t="s">
+      <c r="DX2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="DX2" s="2" t="s">
+      <c r="DY2" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="DY2" s="2" t="s">
+      <c r="DZ2" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="DZ2" s="2" t="s">
+      <c r="EA2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="EA2" s="2" t="s">
+      <c r="EB2" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="EB2" s="2" t="s">
+      <c r="EC2" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="EC2" s="2" t="s">
+      <c r="ED2" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="ED2" s="2" t="s">
+      <c r="EE2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="EE2" s="2" t="s">
+      <c r="EF2" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="EF2" s="2" t="s">
+      <c r="EG2" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="EG2" s="2" t="s">
+      <c r="EH2" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="EH2" s="2" t="s">
+      <c r="EI2" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="EI2" s="2" t="s">
+      <c r="EJ2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="EJ2" s="2" t="s">
+      <c r="EK2" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="EK2" s="2" t="s">
+      <c r="EL2" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="EL2" s="2" t="s">
+      <c r="EM2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="EM2" s="2" t="s">
+      <c r="EN2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="EN2" s="2" t="s">
+      <c r="EO2" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="EO2" s="2" t="s">
+      <c r="EP2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="EP2" s="2" t="s">
+      <c r="EQ2" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="EQ2" s="2" t="s">
+      <c r="ER2" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="ER2" s="2" t="s">
+      <c r="ES2" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="ES2" s="2" t="s">
+      <c r="ET2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="ET2" s="2" t="s">
+      <c r="EU2" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="EU2" s="2" t="s">
+      <c r="EV2" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="EV2" s="2" t="s">
+      <c r="EW2" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="EW2" s="2" t="s">
+      <c r="EX2" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="EX2" s="2" t="s">
+      <c r="EY2" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="EY2" s="2" t="s">
+      <c r="EZ2" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="EZ2" s="2" t="s">
+      <c r="FA2" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="FA2" s="2" t="s">
+      <c r="FB2" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="FB2" s="2" t="s">
+      <c r="FC2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="FC2" s="2" t="s">
+      <c r="FD2" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="FD2" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="FE2" s="2" t="s">
         <v>226</v>
       </c>
       <c r="FF2" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="FG2" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="FG2" s="2" t="s">
+      <c r="FH2" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="FH2" s="2" t="s">
+      <c r="FI2" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="FI2" s="3"/>
+      <c r="FJ2" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="42">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2 I2:J2 L2:T2 Y2:AE2 AI2 AL2:AM2 AP2 AS2 AV2 AY2 BB2 BJ2 BQ2 BY2:CC2 DD2:DE2 DG2:DH2 DL2:DO2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2 I2:J2 L2:U2 Z2:AF2 AJ2 AM2:AN2 AQ2 AT2 AW2 AZ2 BC2 BK2 BR2 BZ2:CD2 DE2:DF2 DH2:DI2 DM2:DP2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2 AF2 BX2 CI2 EW2 EZ2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:X2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2 AG2 BY2 CJ2 EX2 FA2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:Y2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Tidak sama sekali,Kurang dari 1 minggu,Lebih dari 1 minggu,Hampir setiap hari"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"1 s.d &lt;10 tahun lalu,10 s.d &lt;15 tahun lalu,15 tahun lalu atau lebih"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2 BI2 BO2:BP2 BW2 CE2 CJ2 CM2 CP2 CR2 DC2 DF2 DI2 DP2 DR2 DW2 DZ2 ED2 EI2 EL2 EO2 ES2 FB2 FG2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2 BJ2 BP2:BQ2 BX2 CF2 CK2 CN2 CQ2 CS2 DD2 DG2 DJ2 DQ2 DS2 DX2 EA2 EE2 EJ2 EM2 EP2 ET2 FC2 FH2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2 FC2:FF2 FH2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2 FD2:FG2 FI2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DK2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DK2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EV2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EV2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EX2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EY2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EY2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EZ2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FA2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="FB2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
wip skilas mobilisasi skilas malnutrisi skilas depresi
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA5E5AC-197F-8443-A79D-1847612006D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49439FB0-E9BA-8D43-9787-EB1265CC9BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -708,7 +708,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="255">
   <si>
     <t>batas_awal</t>
   </si>
@@ -1455,6 +1455,24 @@
   </si>
   <si>
     <t>ulangi_3_kata_sebelumnya</t>
+  </si>
+  <si>
+    <t>berdiri_di_kursi</t>
+  </si>
+  <si>
+    <t>berat_badan_berkurang</t>
+  </si>
+  <si>
+    <t>hilang_nafsu_makan</t>
+  </si>
+  <si>
+    <t>lila_kurang_21cm</t>
+  </si>
+  <si>
+    <t>2_minggu_terakhir_sedih</t>
+  </si>
+  <si>
+    <t>2_minggu_sedikit_minat</t>
   </si>
 </sst>
 </file>
@@ -1830,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FW4"/>
+  <dimension ref="A1:GC4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1986,9 +2004,15 @@
     <col min="177" max="177" width="16" bestFit="1" customWidth="1"/>
     <col min="178" max="178" width="21" bestFit="1" customWidth="1"/>
     <col min="179" max="179" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="180" max="180" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="181" max="181" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="18" bestFit="1" customWidth="1"/>
+    <col min="183" max="183" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="184" max="184" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="185" max="185" width="21.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:179" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:185" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2526,8 +2550,26 @@
       <c r="FW1" s="1" t="s">
         <v>248</v>
       </c>
+      <c r="FX1" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="FY1" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="FZ1" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="GA1" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="GB1" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="GC1" s="1" t="s">
+        <v>254</v>
+      </c>
     </row>
-    <row r="2" spans="1:179" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:185" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -3046,7 +3088,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="3" spans="1:179" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:185" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>176</v>
       </c>
@@ -3565,7 +3607,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:179" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:185" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>176</v>
       </c>
@@ -3706,13 +3748,31 @@
       <c r="FW4" t="s">
         <v>180</v>
       </c>
+      <c r="FX4" t="s">
+        <v>180</v>
+      </c>
+      <c r="FY4" t="s">
+        <v>180</v>
+      </c>
+      <c r="FZ4" t="s">
+        <v>180</v>
+      </c>
+      <c r="GA4" t="s">
+        <v>180</v>
+      </c>
+      <c r="GB4" t="s">
+        <v>180</v>
+      </c>
+      <c r="GC4" t="s">
+        <v>180</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="48">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Belum Menikah,Menikah,Cerai Mati,Cerai Hidup"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G4 I2:J4 L2:U4 Z2:AF4 AJ2:AJ4 AM2:AN4 AQ2:AQ4 AT2:AT4 AW2:AW4 AZ2:AZ4 BC2:BC4 BK2:BK4 BR2:BR4 BZ2:CD4 DE2:DF4 DH2:DI4 DM2:DP4 EQ2:ET4 FU2:FU4 FW2:FW4" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G4 I2:J4 L2:U4 Z2:AF4 AJ2:AJ4 AM2:AN4 AQ2:AQ4 AT2:AT4 AW2:AW4 AZ2:AZ4 BC2:BC4 BK2:BK4 BR2:BR4 BZ2:CD4 DE2:DF4 DH2:DI4 DM2:DP4 EQ2:ET4 FU2:FU4 FW2:GC4" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{00000000-0002-0000-0000-000002000000}">

</xml_diff>

<commit_message>
wip modularisasi skining mandiri
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -732,7 +732,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:GH4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="GH2" t="inlineStr">
         <is>
-          <t>FAILED: name 'ScreeningDemografi' is not defined</t>
+          <t>FAILED: name 'page' is not defined</t>
         </is>
       </c>
     </row>
@@ -3513,6 +3513,11 @@
       <c r="FT3" s="2" t="inlineStr">
         <is>
           <t>Reaktif</t>
+        </is>
+      </c>
+      <c r="GH3" t="inlineStr">
+        <is>
+          <t>FAILED: name 'do_demografi_dewasa_perempuan' is not defined</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip modularisasi skining nakes
</commit_message>
<xml_diff>
--- a/dataset/pelayanan.xlsx
+++ b/dataset/pelayanan.xlsx
@@ -2681,7 +2681,7 @@
       </c>
       <c r="GH2" t="inlineStr">
         <is>
-          <t>FAILED: name 'page' is not defined</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="GH3" t="inlineStr">
         <is>
-          <t>FAILED: name 'do_demografi_dewasa_perempuan' is not defined</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -3723,6 +3723,14 @@
           <t>Tergantung pertolongan orang lain</t>
         </is>
       </c>
+      <c r="GH4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAILED: Page.goto: net::ERR_ABORTED at https://sehatindonesiaku.kemkes.go.id/ckg-pelayanan
+Call log:
+  - navigating to "https://sehatindonesiaku.kemkes.go.id/ckg-pelayanan", waiting until "load"
+</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="52">

</xml_diff>